<commit_message>
feat: simplify annotation occurrence authoring
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/content/authoring/templates/ignite-materialset-workbook-v1.xlsx
+++ b/content/authoring/templates/ignite-materialset-workbook-v1.xlsx
@@ -107,7 +107,7 @@
     <t>Annotations</t>
   </si>
   <si>
-    <t>Required: type, strategy, and a card locator (cardNumber or cardId). Phase 2A.1 strategy is phraseOccurrence with phrase + 1-based occurrenceIndex. Types listed below are SYNTHETIC/DEV vocabulary, not official committee notation. Official mapping is Phase 2B.</t>
+    <t>Required: type, strategy, and a card locator (cardNumber or cardId). For phraseOccurrence, type the exact phrase from the verse. occurrenceIndex is optional when that exact phrase occurs once — leave it blank. If the phrase occurs more than once, enter the 1-based occurrence number (1, 2, 3, …) for the match you mean. The tool will not guess. Types listed below are SYNTHETIC/DEV vocabulary, not official committee notation. Official mapping is Phase 2B.</t>
   </si>
   <si>
     <t>Synthetic annotation types</t>
@@ -736,7 +736,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" ht="72" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>

</xml_diff>